<commit_message>
New and improved panel-CLI!
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/order_archive/Casa/Casa_Bakery_20260316.xlsx
+++ b/WorkBot/main/data/order_archive/Casa/Casa_Bakery_20260316.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,13 +455,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
         <v>27.42</v>
       </c>
       <c r="E2" t="n">
-        <v>164.52</v>
+        <v>246.78</v>
       </c>
     </row>
     <row r="3">
@@ -476,34 +476,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
         <v>94.13</v>
       </c>
       <c r="E3" t="n">
-        <v>564.78</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>52012</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flour - Rice</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>31.05</v>
-      </c>
-      <c r="E4" t="n">
-        <v>31.05</v>
+        <v>658.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>